<commit_message>
modify test data (registration)BasePage and created Registration Page
</commit_message>
<xml_diff>
--- a/ testdata/register_user.xlsx
+++ b/ testdata/register_user.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SeleniumLearning\LambdatestPlayground\ testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F670B0DE-565A-47BA-80C2-78BE18F43551}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F4F2F56-B6C8-4483-AA39-9DC667747F55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A74BF28C-13B3-448C-A368-528222B83AEA}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="25">
   <si>
     <t>hafiz@gmail.com</t>
   </si>
@@ -110,10 +110,7 @@
     <t>PrivacyPolicy</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>No</t>
+    <t xml:space="preserve">false </t>
   </si>
 </sst>
 </file>
@@ -608,11 +605,11 @@
       <c r="F2" s="4">
         <v>123456</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>24</v>
+      <c r="G2" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>4</v>
@@ -635,10 +632,10 @@
         <v>123457</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H3" s="4" t="s">
         <v>24</v>
+      </c>
+      <c r="H3" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>4</v>
@@ -661,11 +658,11 @@
       <c r="F4" s="4">
         <v>123458</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>25</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>4</v>
@@ -688,11 +685,11 @@
       <c r="F5" s="4">
         <v>123459</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>24</v>
+      <c r="G5" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>4</v>
@@ -716,10 +713,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>4</v>
@@ -742,11 +739,11 @@
         <v>9</v>
       </c>
       <c r="F7" s="5"/>
-      <c r="G7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>24</v>
+      <c r="G7" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>4</v>
@@ -775,7 +772,7 @@
         <v>24</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>4</v>
@@ -800,11 +797,11 @@
       <c r="F9" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>24</v>
+      <c r="G9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="b">
+        <v>1</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>3</v>

</xml_diff>